<commit_message>
update dependency and analysis schemas
</commit_message>
<xml_diff>
--- a/inst/resources/dependency_schema_data_household_template.xlsx
+++ b/inst/resources/dependency_schema_data_household_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acted-my.sharepoint.com/personal/martina_vit_impact-initiatives_org/Documents/public_health_resources/inst/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{CF71D149-0280-40DA-9004-7ADEC66A4EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E7BF2F7-7EC9-4BEF-A60C-F2EB88796888}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{CF71D149-0280-40DA-9004-7ADEC66A4EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E82E33B5-7874-42A4-BBD5-963CB5A88397}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$390</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
 </workbook>
 </file>
 
@@ -4139,19 +4139,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H390"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.54296875" customWidth="1"/>
-    <col min="2" max="2" width="37.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="69.86328125" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="37.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.85546875" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="62" customWidth="1"/>
-    <col min="6" max="6" width="17.7265625" customWidth="1"/>
-    <col min="7" max="7" width="5.40625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.40625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4177,7 +4177,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4217,7 +4217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4237,7 +4237,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4277,7 +4277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4297,7 +4297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -4317,7 +4317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -4337,7 +4337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -4357,7 +4357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4377,7 +4377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -4397,7 +4397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -4437,7 +4437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -4457,7 +4457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -4477,7 +4477,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -4497,7 +4497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -4517,7 +4517,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -4537,7 +4537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -4557,7 +4557,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -4577,7 +4577,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -4617,7 +4617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -4677,7 +4677,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -4697,7 +4697,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -4717,7 +4717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -4757,7 +4757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -4777,7 +4777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -4797,7 +4797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -4817,7 +4817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -4837,7 +4837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -4857,7 +4857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -4877,7 +4877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -4897,7 +4897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -4917,7 +4917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -4937,7 +4937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>8</v>
       </c>
@@ -4957,7 +4957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -4977,7 +4977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -4997,7 +4997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>8</v>
       </c>
@@ -5017,7 +5017,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>8</v>
       </c>
@@ -5037,7 +5037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -5057,7 +5057,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>8</v>
       </c>
@@ -5077,7 +5077,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -5097,7 +5097,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -5117,7 +5117,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -5137,7 +5137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>8</v>
       </c>
@@ -5157,7 +5157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>8</v>
       </c>
@@ -5177,7 +5177,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>8</v>
       </c>
@@ -5197,7 +5197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -5237,7 +5237,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>8</v>
       </c>
@@ -5257,7 +5257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -5277,7 +5277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>8</v>
       </c>
@@ -5297,7 +5297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>8</v>
       </c>
@@ -5317,7 +5317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -5337,7 +5337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>8</v>
       </c>
@@ -5357,7 +5357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>8</v>
       </c>
@@ -5377,7 +5377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -5397,7 +5397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -5417,7 +5417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -5437,7 +5437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -5457,7 +5457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>8</v>
       </c>
@@ -5477,7 +5477,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>8</v>
       </c>
@@ -5497,7 +5497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>8</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>8</v>
       </c>
@@ -5537,7 +5537,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>8</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -5577,7 +5577,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>8</v>
       </c>
@@ -5597,7 +5597,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>8</v>
       </c>
@@ -5617,7 +5617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>8</v>
       </c>
@@ -5637,7 +5637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -5657,7 +5657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -5677,7 +5677,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -5697,7 +5697,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -5717,7 +5717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -5737,7 +5737,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -5757,7 +5757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -5777,7 +5777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>8</v>
       </c>
@@ -5797,7 +5797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>8</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>8</v>
       </c>
@@ -5837,7 +5837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -5857,7 +5857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>8</v>
       </c>
@@ -5877,7 +5877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>8</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -5917,7 +5917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -5937,7 +5937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>8</v>
       </c>
@@ -5957,7 +5957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -5977,7 +5977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>8</v>
       </c>
@@ -5997,7 +5997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -6017,7 +6017,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>8</v>
       </c>
@@ -6037,7 +6037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>8</v>
       </c>
@@ -6057,7 +6057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>8</v>
       </c>
@@ -6077,7 +6077,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>8</v>
       </c>
@@ -6097,7 +6097,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>8</v>
       </c>
@@ -6117,7 +6117,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>8</v>
       </c>
@@ -6137,7 +6137,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>8</v>
       </c>
@@ -6157,7 +6157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>8</v>
       </c>
@@ -6177,7 +6177,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>8</v>
       </c>
@@ -6197,7 +6197,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>8</v>
       </c>
@@ -6217,7 +6217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>8</v>
       </c>
@@ -6237,7 +6237,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>8</v>
       </c>
@@ -6257,7 +6257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>8</v>
       </c>
@@ -6277,7 +6277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>8</v>
       </c>
@@ -6297,7 +6297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>8</v>
       </c>
@@ -6317,7 +6317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>8</v>
       </c>
@@ -6337,7 +6337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>8</v>
       </c>
@@ -6357,7 +6357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>8</v>
       </c>
@@ -6377,7 +6377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>8</v>
       </c>
@@ -6397,7 +6397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>8</v>
       </c>
@@ -6417,7 +6417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>8</v>
       </c>
@@ -6437,7 +6437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>8</v>
       </c>
@@ -6457,7 +6457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>8</v>
       </c>
@@ -6477,7 +6477,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>8</v>
       </c>
@@ -6497,7 +6497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>8</v>
       </c>
@@ -6517,7 +6517,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>8</v>
       </c>
@@ -6537,7 +6537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>8</v>
       </c>
@@ -6557,7 +6557,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>8</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>8</v>
       </c>
@@ -6597,7 +6597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>8</v>
       </c>
@@ -6617,7 +6617,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>8</v>
       </c>
@@ -6637,7 +6637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>8</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>8</v>
       </c>
@@ -6677,7 +6677,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>8</v>
       </c>
@@ -6697,7 +6697,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>8</v>
       </c>
@@ -6717,7 +6717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>8</v>
       </c>
@@ -6737,7 +6737,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>8</v>
       </c>
@@ -6757,7 +6757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>8</v>
       </c>
@@ -6777,7 +6777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>8</v>
       </c>
@@ -6797,7 +6797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>8</v>
       </c>
@@ -6817,7 +6817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>8</v>
       </c>
@@ -6837,7 +6837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>8</v>
       </c>
@@ -6857,7 +6857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>8</v>
       </c>
@@ -6877,7 +6877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>8</v>
       </c>
@@ -6897,7 +6897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>8</v>
       </c>
@@ -6917,7 +6917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>8</v>
       </c>
@@ -6937,7 +6937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>8</v>
       </c>
@@ -6957,7 +6957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>8</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>8</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>8</v>
       </c>
@@ -7017,7 +7017,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>8</v>
       </c>
@@ -7037,7 +7037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>8</v>
       </c>
@@ -7057,7 +7057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>8</v>
       </c>
@@ -7077,7 +7077,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>8</v>
       </c>
@@ -7097,7 +7097,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>8</v>
       </c>
@@ -7117,7 +7117,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>8</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>8</v>
       </c>
@@ -7157,7 +7157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>8</v>
       </c>
@@ -7177,7 +7177,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>8</v>
       </c>
@@ -7197,7 +7197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>8</v>
       </c>
@@ -7217,7 +7217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>8</v>
       </c>
@@ -7237,7 +7237,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>8</v>
       </c>
@@ -7257,7 +7257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>8</v>
       </c>
@@ -7277,7 +7277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>8</v>
       </c>
@@ -7297,7 +7297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>8</v>
       </c>
@@ -7317,7 +7317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>8</v>
       </c>
@@ -7337,7 +7337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>8</v>
       </c>
@@ -7357,7 +7357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>8</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>8</v>
       </c>
@@ -7397,7 +7397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>8</v>
       </c>
@@ -7417,7 +7417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>8</v>
       </c>
@@ -7437,7 +7437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>8</v>
       </c>
@@ -7457,7 +7457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>8</v>
       </c>
@@ -7477,7 +7477,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>8</v>
       </c>
@@ -7497,7 +7497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>8</v>
       </c>
@@ -7517,7 +7517,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>8</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>8</v>
       </c>
@@ -7557,7 +7557,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>8</v>
       </c>
@@ -7577,7 +7577,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>8</v>
       </c>
@@ -7597,7 +7597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>8</v>
       </c>
@@ -7617,7 +7617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>8</v>
       </c>
@@ -7637,7 +7637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>8</v>
       </c>
@@ -7657,7 +7657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>8</v>
       </c>
@@ -7677,7 +7677,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>8</v>
       </c>
@@ -7697,7 +7697,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>8</v>
       </c>
@@ -7717,7 +7717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>8</v>
       </c>
@@ -7737,7 +7737,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>8</v>
       </c>
@@ -7757,7 +7757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>8</v>
       </c>
@@ -7777,7 +7777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>8</v>
       </c>
@@ -7797,7 +7797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>8</v>
       </c>
@@ -7817,7 +7817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>8</v>
       </c>
@@ -7837,7 +7837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>8</v>
       </c>
@@ -7857,7 +7857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>8</v>
       </c>
@@ -7877,7 +7877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>8</v>
       </c>
@@ -7897,7 +7897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>8</v>
       </c>
@@ -7917,7 +7917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>8</v>
       </c>
@@ -7937,7 +7937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>8</v>
       </c>
@@ -7957,7 +7957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>8</v>
       </c>
@@ -7977,7 +7977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>8</v>
       </c>
@@ -7997,7 +7997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>8</v>
       </c>
@@ -8017,7 +8017,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>8</v>
       </c>
@@ -8037,7 +8037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>8</v>
       </c>
@@ -8057,7 +8057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>8</v>
       </c>
@@ -8077,7 +8077,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>8</v>
       </c>
@@ -8097,7 +8097,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>8</v>
       </c>
@@ -8117,7 +8117,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>8</v>
       </c>
@@ -8137,7 +8137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>8</v>
       </c>
@@ -8157,7 +8157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>8</v>
       </c>
@@ -8177,7 +8177,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>8</v>
       </c>
@@ -8197,7 +8197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>8</v>
       </c>
@@ -8217,7 +8217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>8</v>
       </c>
@@ -8237,7 +8237,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>8</v>
       </c>
@@ -8257,7 +8257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>8</v>
       </c>
@@ -8277,7 +8277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>8</v>
       </c>
@@ -8297,7 +8297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>8</v>
       </c>
@@ -8317,7 +8317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>8</v>
       </c>
@@ -8337,7 +8337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>8</v>
       </c>
@@ -8357,7 +8357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>8</v>
       </c>
@@ -8377,7 +8377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>8</v>
       </c>
@@ -8397,7 +8397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>8</v>
       </c>
@@ -8417,7 +8417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>8</v>
       </c>
@@ -8437,7 +8437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>8</v>
       </c>
@@ -8457,7 +8457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>8</v>
       </c>
@@ -8477,7 +8477,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>8</v>
       </c>
@@ -8497,7 +8497,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>8</v>
       </c>
@@ -8517,7 +8517,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>8</v>
       </c>
@@ -8537,7 +8537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>8</v>
       </c>
@@ -8557,7 +8557,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>8</v>
       </c>
@@ -8577,7 +8577,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>8</v>
       </c>
@@ -8597,7 +8597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>8</v>
       </c>
@@ -8617,7 +8617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>8</v>
       </c>
@@ -8637,7 +8637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>8</v>
       </c>
@@ -8657,7 +8657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>8</v>
       </c>
@@ -8677,7 +8677,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>8</v>
       </c>
@@ -8697,7 +8697,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>8</v>
       </c>
@@ -8717,7 +8717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>8</v>
       </c>
@@ -8737,7 +8737,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>8</v>
       </c>
@@ -8757,7 +8757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>8</v>
       </c>
@@ -8777,7 +8777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>8</v>
       </c>
@@ -8797,7 +8797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>8</v>
       </c>
@@ -8817,7 +8817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>8</v>
       </c>
@@ -8837,7 +8837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>8</v>
       </c>
@@ -8857,7 +8857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>8</v>
       </c>
@@ -8877,7 +8877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>8</v>
       </c>
@@ -8897,7 +8897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>8</v>
       </c>
@@ -8917,7 +8917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>8</v>
       </c>
@@ -8937,7 +8937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>8</v>
       </c>
@@ -8957,7 +8957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>8</v>
       </c>
@@ -8977,7 +8977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>8</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>8</v>
       </c>
@@ -9017,7 +9017,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>8</v>
       </c>
@@ -9037,7 +9037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>8</v>
       </c>
@@ -9057,7 +9057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>8</v>
       </c>
@@ -9077,7 +9077,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>8</v>
       </c>
@@ -9097,7 +9097,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>8</v>
       </c>
@@ -9117,7 +9117,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>8</v>
       </c>
@@ -9137,7 +9137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>8</v>
       </c>
@@ -9157,7 +9157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>8</v>
       </c>
@@ -9177,7 +9177,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>8</v>
       </c>
@@ -9197,7 +9197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>8</v>
       </c>
@@ -9217,7 +9217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>8</v>
       </c>
@@ -9237,7 +9237,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>8</v>
       </c>
@@ -9257,7 +9257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>8</v>
       </c>
@@ -9277,7 +9277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>8</v>
       </c>
@@ -9297,7 +9297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>8</v>
       </c>
@@ -9317,7 +9317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>8</v>
       </c>
@@ -9337,7 +9337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>8</v>
       </c>
@@ -9357,7 +9357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>8</v>
       </c>
@@ -9377,7 +9377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>8</v>
       </c>
@@ -9397,7 +9397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>8</v>
       </c>
@@ -9417,7 +9417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>8</v>
       </c>
@@ -9437,7 +9437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>8</v>
       </c>
@@ -9457,7 +9457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>8</v>
       </c>
@@ -9477,7 +9477,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>8</v>
       </c>
@@ -9497,7 +9497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>8</v>
       </c>
@@ -9517,7 +9517,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>8</v>
       </c>
@@ -9537,7 +9537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>8</v>
       </c>
@@ -9557,7 +9557,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>8</v>
       </c>
@@ -9577,7 +9577,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>8</v>
       </c>
@@ -9597,7 +9597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>8</v>
       </c>
@@ -9617,7 +9617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>8</v>
       </c>
@@ -9637,7 +9637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>8</v>
       </c>
@@ -9657,7 +9657,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>8</v>
       </c>
@@ -9677,7 +9677,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>8</v>
       </c>
@@ -9697,7 +9697,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>8</v>
       </c>
@@ -9717,7 +9717,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>8</v>
       </c>
@@ -9737,7 +9737,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>8</v>
       </c>
@@ -9757,7 +9757,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>8</v>
       </c>
@@ -9777,7 +9777,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>8</v>
       </c>
@@ -9797,7 +9797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>8</v>
       </c>
@@ -9817,7 +9817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>8</v>
       </c>
@@ -9837,7 +9837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>8</v>
       </c>
@@ -9857,7 +9857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>8</v>
       </c>
@@ -9877,7 +9877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>8</v>
       </c>
@@ -9897,7 +9897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>8</v>
       </c>
@@ -9917,7 +9917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>8</v>
       </c>
@@ -9937,7 +9937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>8</v>
       </c>
@@ -9957,7 +9957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>8</v>
       </c>
@@ -9977,7 +9977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>8</v>
       </c>
@@ -9997,7 +9997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>8</v>
       </c>
@@ -10017,7 +10017,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>8</v>
       </c>
@@ -10037,7 +10037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>8</v>
       </c>
@@ -10057,7 +10057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>8</v>
       </c>
@@ -10077,7 +10077,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>8</v>
       </c>
@@ -10097,7 +10097,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>8</v>
       </c>
@@ -10117,7 +10117,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>8</v>
       </c>
@@ -10137,7 +10137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>8</v>
       </c>
@@ -10157,7 +10157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>8</v>
       </c>
@@ -10177,7 +10177,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>8</v>
       </c>
@@ -10197,7 +10197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>8</v>
       </c>
@@ -10217,7 +10217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>8</v>
       </c>
@@ -10237,7 +10237,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>8</v>
       </c>
@@ -10257,7 +10257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>8</v>
       </c>
@@ -10277,7 +10277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>8</v>
       </c>
@@ -10297,7 +10297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>8</v>
       </c>
@@ -10317,7 +10317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>8</v>
       </c>
@@ -10337,7 +10337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>8</v>
       </c>
@@ -10357,7 +10357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>8</v>
       </c>
@@ -10377,7 +10377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>8</v>
       </c>
@@ -10397,7 +10397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>8</v>
       </c>
@@ -10417,7 +10417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>8</v>
       </c>
@@ -10437,7 +10437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>8</v>
       </c>
@@ -10457,7 +10457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>8</v>
       </c>
@@ -10477,7 +10477,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>8</v>
       </c>
@@ -10497,7 +10497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>8</v>
       </c>
@@ -10517,7 +10517,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>8</v>
       </c>
@@ -10537,7 +10537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>8</v>
       </c>
@@ -10557,7 +10557,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>8</v>
       </c>
@@ -10577,7 +10577,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>8</v>
       </c>
@@ -10597,7 +10597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>8</v>
       </c>
@@ -10617,7 +10617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="324" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>8</v>
       </c>
@@ -10637,7 +10637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>8</v>
       </c>
@@ -10657,7 +10657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="326" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="326" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>8</v>
       </c>
@@ -10677,7 +10677,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="327" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>8</v>
       </c>
@@ -10697,7 +10697,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="328" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>8</v>
       </c>
@@ -10717,7 +10717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="329" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>8</v>
       </c>
@@ -10737,7 +10737,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="330" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="330" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>8</v>
       </c>
@@ -10757,7 +10757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="331" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>8</v>
       </c>
@@ -10777,7 +10777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="332" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>8</v>
       </c>
@@ -10797,7 +10797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="333" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>8</v>
       </c>
@@ -10817,7 +10817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="334" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>8</v>
       </c>
@@ -10837,7 +10837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="335" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>8</v>
       </c>
@@ -10857,7 +10857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="336" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>8</v>
       </c>
@@ -10877,7 +10877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="337" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>8</v>
       </c>
@@ -10897,7 +10897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="338" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>8</v>
       </c>
@@ -10917,7 +10917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="339" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="339" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>8</v>
       </c>
@@ -10937,7 +10937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="340" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="340" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>8</v>
       </c>
@@ -10957,7 +10957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="341" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>8</v>
       </c>
@@ -10977,7 +10977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="342" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>8</v>
       </c>
@@ -10997,7 +10997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="343" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="343" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>8</v>
       </c>
@@ -11017,7 +11017,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="344" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>8</v>
       </c>
@@ -11037,7 +11037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="345" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>8</v>
       </c>
@@ -11057,7 +11057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="346" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="346" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>8</v>
       </c>
@@ -11077,7 +11077,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="347" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="347" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>8</v>
       </c>
@@ -11097,7 +11097,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="348" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>8</v>
       </c>
@@ -11117,7 +11117,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="349" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>8</v>
       </c>
@@ -11137,7 +11137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="350" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="350" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>8</v>
       </c>
@@ -11157,7 +11157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="351" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>8</v>
       </c>
@@ -11177,7 +11177,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="352" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>8</v>
       </c>
@@ -11197,7 +11197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="353" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="353" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>8</v>
       </c>
@@ -11217,7 +11217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="354" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="354" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>8</v>
       </c>
@@ -11237,7 +11237,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="355" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="355" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>8</v>
       </c>
@@ -11257,7 +11257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="356" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="356" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>8</v>
       </c>
@@ -11277,7 +11277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="357" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="357" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>8</v>
       </c>
@@ -11297,7 +11297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="358" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="358" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>8</v>
       </c>
@@ -11317,7 +11317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="359" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="359" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>8</v>
       </c>
@@ -11337,7 +11337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="360" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="360" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>8</v>
       </c>
@@ -11357,7 +11357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="361" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="361" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>8</v>
       </c>
@@ -11377,7 +11377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="362" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="362" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>8</v>
       </c>
@@ -11397,7 +11397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="363" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="363" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>8</v>
       </c>
@@ -11417,7 +11417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="364" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="364" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>8</v>
       </c>
@@ -11437,7 +11437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="365" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="365" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
         <v>8</v>
       </c>
@@ -11457,7 +11457,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="366" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="366" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
         <v>8</v>
       </c>
@@ -11477,7 +11477,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="367" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="367" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
         <v>8</v>
       </c>
@@ -11497,7 +11497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="368" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="368" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
         <v>8</v>
       </c>
@@ -11517,7 +11517,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="369" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="369" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
         <v>8</v>
       </c>
@@ -11537,7 +11537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="370" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="370" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
         <v>8</v>
       </c>
@@ -11557,7 +11557,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="371" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="371" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
         <v>8</v>
       </c>
@@ -11577,7 +11577,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="372" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="372" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
         <v>8</v>
       </c>
@@ -11597,7 +11597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="373" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="373" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
         <v>8</v>
       </c>
@@ -11617,7 +11617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="374" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="374" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
         <v>8</v>
       </c>
@@ -11637,7 +11637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="375" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="375" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
         <v>8</v>
       </c>
@@ -11657,7 +11657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="376" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="376" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
         <v>8</v>
       </c>
@@ -11677,7 +11677,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="377" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="377" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
         <v>8</v>
       </c>
@@ -11697,7 +11697,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="378" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="378" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
         <v>8</v>
       </c>
@@ -11717,7 +11717,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="379" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="379" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
         <v>8</v>
       </c>
@@ -11737,7 +11737,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="380" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="380" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
         <v>8</v>
       </c>
@@ -11757,7 +11757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="381" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="381" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
         <v>8</v>
       </c>
@@ -11777,7 +11777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="382" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="382" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
         <v>8</v>
       </c>
@@ -11797,7 +11797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="383" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="383" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
         <v>8</v>
       </c>
@@ -11817,7 +11817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="384" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="384" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
         <v>8</v>
       </c>
@@ -11837,7 +11837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="385" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="385" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
         <v>8</v>
       </c>
@@ -11857,7 +11857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="386" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="386" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
         <v>8</v>
       </c>
@@ -11877,7 +11877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="387" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="387" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
         <v>8</v>
       </c>
@@ -11897,7 +11897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="388" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="388" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
         <v>8</v>
       </c>
@@ -11917,7 +11917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="389" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="389" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
         <v>8</v>
       </c>
@@ -11937,7 +11937,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="390" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="390" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
         <v>8</v>
       </c>

</xml_diff>